<commit_message>
plan: cập nhật trạng thái/% 46 task P0 (35 xong, 6 đang làm, 5 bị chặn do cần tài khoản/hạ tầng)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NQGF9iU7jMGkJMH1PrJV2s
</commit_message>
<xml_diff>
--- a/docs/plan/QuickAssist_KeHoach_PhanCong_v2.xlsx
+++ b/docs/plan/QuickAssist_KeHoach_PhanCong_v2.xlsx
@@ -3801,11 +3801,13 @@
       <c r="M4" s="3" t="s">
         <v>185</v>
       </c>
-      <c r="N4" s="3" t="s">
-        <v>186</v>
+      <c r="N4" s="3" t="inlineStr">
+        <is>
+          <t>Đang thực hiện</t>
+        </is>
       </c>
       <c r="O4" s="9" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
       <c r="P4" s="10" t="s">
         <v>187</v>
@@ -3851,11 +3853,13 @@
       <c r="M5" s="3" t="s">
         <v>192</v>
       </c>
-      <c r="N5" s="3" t="s">
-        <v>186</v>
+      <c r="N5" s="3" t="inlineStr">
+        <is>
+          <t>Đã hoàn thành</t>
+        </is>
       </c>
       <c r="O5" s="9" t="n">
-        <v>0.7</v>
+        <v>1.0</v>
       </c>
       <c r="P5" s="10" t="s">
         <v>193</v>
@@ -3901,11 +3905,13 @@
       <c r="M6" s="3" t="s">
         <v>198</v>
       </c>
-      <c r="N6" s="3" t="s">
-        <v>199</v>
+      <c r="N6" s="3" t="inlineStr">
+        <is>
+          <t>Bị chặn</t>
+        </is>
       </c>
       <c r="O6" s="9" t="n">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="P6" s="10" t="s">
         <v>200</v>
@@ -3951,11 +3957,13 @@
       <c r="M7" s="3" t="s">
         <v>205</v>
       </c>
-      <c r="N7" s="3" t="s">
-        <v>199</v>
+      <c r="N7" s="3" t="inlineStr">
+        <is>
+          <t>Đã hoàn thành</t>
+        </is>
       </c>
       <c r="O7" s="9" t="n">
-        <v>0</v>
+        <v>1.0</v>
       </c>
       <c r="P7" s="10" t="s">
         <v>206</v>
@@ -4001,11 +4009,13 @@
       <c r="M8" s="3" t="s">
         <v>212</v>
       </c>
-      <c r="N8" s="3" t="s">
-        <v>186</v>
+      <c r="N8" s="3" t="inlineStr">
+        <is>
+          <t>Đang thực hiện</t>
+        </is>
       </c>
       <c r="O8" s="9" t="n">
-        <v>0.7</v>
+        <v>0.9</v>
       </c>
       <c r="P8" s="10" t="s">
         <v>213</v>
@@ -4051,11 +4061,13 @@
       <c r="M9" s="3" t="s">
         <v>218</v>
       </c>
-      <c r="N9" s="3" t="s">
-        <v>186</v>
+      <c r="N9" s="3" t="inlineStr">
+        <is>
+          <t>Đang thực hiện</t>
+        </is>
       </c>
       <c r="O9" s="9" t="n">
-        <v>0.7</v>
+        <v>0.9</v>
       </c>
       <c r="P9" s="10" t="s">
         <v>219</v>
@@ -4101,11 +4113,13 @@
       <c r="M10" s="3" t="s">
         <v>223</v>
       </c>
-      <c r="N10" s="3" t="s">
-        <v>186</v>
+      <c r="N10" s="3" t="inlineStr">
+        <is>
+          <t>Đã hoàn thành</t>
+        </is>
       </c>
       <c r="O10" s="9" t="n">
-        <v>0.6</v>
+        <v>1.0</v>
       </c>
       <c r="P10" s="10" t="s">
         <v>200</v>
@@ -4151,11 +4165,13 @@
       <c r="M11" s="3" t="s">
         <v>228</v>
       </c>
-      <c r="N11" s="3" t="s">
-        <v>199</v>
+      <c r="N11" s="3" t="inlineStr">
+        <is>
+          <t>Đã hoàn thành</t>
+        </is>
       </c>
       <c r="O11" s="9" t="n">
-        <v>0</v>
+        <v>1.0</v>
       </c>
       <c r="P11" s="10" t="s">
         <v>229</v>
@@ -4201,11 +4217,13 @@
       <c r="M12" s="3" t="s">
         <v>234</v>
       </c>
-      <c r="N12" s="3" t="s">
-        <v>186</v>
+      <c r="N12" s="3" t="inlineStr">
+        <is>
+          <t>Bị chặn</t>
+        </is>
       </c>
       <c r="O12" s="9" t="n">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="P12" s="10" t="s">
         <v>235</v>
@@ -4251,11 +4269,13 @@
       <c r="M13" s="3" t="s">
         <v>240</v>
       </c>
-      <c r="N13" s="3" t="s">
-        <v>199</v>
+      <c r="N13" s="3" t="inlineStr">
+        <is>
+          <t>Đã hoàn thành</t>
+        </is>
       </c>
       <c r="O13" s="9" t="n">
-        <v>0</v>
+        <v>1.0</v>
       </c>
       <c r="P13" s="10" t="s">
         <v>241</v>
@@ -4301,11 +4321,13 @@
       <c r="M14" s="3" t="s">
         <v>246</v>
       </c>
-      <c r="N14" s="3" t="s">
-        <v>186</v>
+      <c r="N14" s="3" t="inlineStr">
+        <is>
+          <t>Đã hoàn thành</t>
+        </is>
       </c>
       <c r="O14" s="9" t="n">
-        <v>0.6</v>
+        <v>1.0</v>
       </c>
       <c r="P14" s="10" t="s">
         <v>247</v>
@@ -4351,11 +4373,13 @@
       <c r="M15" s="3" t="s">
         <v>253</v>
       </c>
-      <c r="N15" s="3" t="s">
-        <v>186</v>
+      <c r="N15" s="3" t="inlineStr">
+        <is>
+          <t>Đã hoàn thành</t>
+        </is>
       </c>
       <c r="O15" s="9" t="n">
-        <v>0.5</v>
+        <v>1.0</v>
       </c>
       <c r="P15" s="10" t="s">
         <v>254</v>
@@ -4401,11 +4425,13 @@
       <c r="M16" s="3" t="s">
         <v>259</v>
       </c>
-      <c r="N16" s="3" t="s">
-        <v>186</v>
+      <c r="N16" s="3" t="inlineStr">
+        <is>
+          <t>Đang thực hiện</t>
+        </is>
       </c>
       <c r="O16" s="9" t="n">
-        <v>0.5</v>
+        <v>0.9</v>
       </c>
       <c r="P16" s="10" t="s">
         <v>260</v>
@@ -4451,11 +4477,13 @@
       <c r="M17" s="3" t="s">
         <v>266</v>
       </c>
-      <c r="N17" s="3" t="s">
-        <v>186</v>
+      <c r="N17" s="3" t="inlineStr">
+        <is>
+          <t>Đã hoàn thành</t>
+        </is>
       </c>
       <c r="O17" s="9" t="n">
-        <v>0.5</v>
+        <v>1.0</v>
       </c>
       <c r="P17" s="10" t="s">
         <v>267</v>
@@ -4501,11 +4529,13 @@
       <c r="M18" s="3" t="s">
         <v>273</v>
       </c>
-      <c r="N18" s="3" t="s">
-        <v>186</v>
+      <c r="N18" s="3" t="inlineStr">
+        <is>
+          <t>Đã hoàn thành</t>
+        </is>
       </c>
       <c r="O18" s="9" t="n">
-        <v>0.3</v>
+        <v>1.0</v>
       </c>
       <c r="P18" s="10" t="s">
         <v>274</v>
@@ -4551,11 +4581,13 @@
       <c r="M19" s="3" t="s">
         <v>277</v>
       </c>
-      <c r="N19" s="3" t="s">
-        <v>186</v>
+      <c r="N19" s="3" t="inlineStr">
+        <is>
+          <t>Đã hoàn thành</t>
+        </is>
       </c>
       <c r="O19" s="9" t="n">
-        <v>0.6</v>
+        <v>1.0</v>
       </c>
       <c r="P19" s="10" t="s">
         <v>278</v>
@@ -4601,11 +4633,13 @@
       <c r="M20" s="3" t="s">
         <v>282</v>
       </c>
-      <c r="N20" s="3" t="s">
-        <v>186</v>
+      <c r="N20" s="3" t="inlineStr">
+        <is>
+          <t>Đã hoàn thành</t>
+        </is>
       </c>
       <c r="O20" s="9" t="n">
-        <v>0.6</v>
+        <v>1.0</v>
       </c>
       <c r="P20" s="10" t="s">
         <v>283</v>
@@ -4651,11 +4685,13 @@
       <c r="M21" s="3" t="s">
         <v>288</v>
       </c>
-      <c r="N21" s="3" t="s">
-        <v>199</v>
+      <c r="N21" s="3" t="inlineStr">
+        <is>
+          <t>Đã hoàn thành</t>
+        </is>
       </c>
       <c r="O21" s="9" t="n">
-        <v>0</v>
+        <v>1.0</v>
       </c>
       <c r="P21" s="10" t="s">
         <v>241</v>
@@ -4701,11 +4737,13 @@
       <c r="M22" s="3" t="s">
         <v>293</v>
       </c>
-      <c r="N22" s="3" t="s">
-        <v>186</v>
+      <c r="N22" s="3" t="inlineStr">
+        <is>
+          <t>Đã hoàn thành</t>
+        </is>
       </c>
       <c r="O22" s="9" t="n">
-        <v>0.6</v>
+        <v>1.0</v>
       </c>
       <c r="P22" s="10" t="s">
         <v>294</v>
@@ -4751,11 +4789,13 @@
       <c r="M23" s="3" t="s">
         <v>299</v>
       </c>
-      <c r="N23" s="3" t="s">
-        <v>186</v>
+      <c r="N23" s="3" t="inlineStr">
+        <is>
+          <t>Đã hoàn thành</t>
+        </is>
       </c>
       <c r="O23" s="9" t="n">
-        <v>0.5</v>
+        <v>1.0</v>
       </c>
       <c r="P23" s="10" t="s">
         <v>300</v>
@@ -4801,11 +4841,13 @@
       <c r="M24" s="3" t="s">
         <v>305</v>
       </c>
-      <c r="N24" s="3" t="s">
-        <v>186</v>
+      <c r="N24" s="3" t="inlineStr">
+        <is>
+          <t>Đã hoàn thành</t>
+        </is>
       </c>
       <c r="O24" s="9" t="n">
-        <v>0.6</v>
+        <v>1.0</v>
       </c>
       <c r="P24" s="10" t="s">
         <v>306</v>
@@ -4851,11 +4893,13 @@
       <c r="M25" s="3" t="s">
         <v>310</v>
       </c>
-      <c r="N25" s="3" t="s">
-        <v>186</v>
+      <c r="N25" s="3" t="inlineStr">
+        <is>
+          <t>Đã hoàn thành</t>
+        </is>
       </c>
       <c r="O25" s="9" t="n">
-        <v>0.3</v>
+        <v>1.0</v>
       </c>
       <c r="P25" s="10" t="s">
         <v>311</v>
@@ -4901,11 +4945,13 @@
       <c r="M26" s="3" t="s">
         <v>316</v>
       </c>
-      <c r="N26" s="3" t="s">
-        <v>186</v>
+      <c r="N26" s="3" t="inlineStr">
+        <is>
+          <t>Đã hoàn thành</t>
+        </is>
       </c>
       <c r="O26" s="9" t="n">
-        <v>0.6</v>
+        <v>1.0</v>
       </c>
       <c r="P26" s="10" t="s">
         <v>317</v>
@@ -4951,11 +4997,13 @@
       <c r="M27" s="3" t="s">
         <v>322</v>
       </c>
-      <c r="N27" s="3" t="s">
-        <v>186</v>
+      <c r="N27" s="3" t="inlineStr">
+        <is>
+          <t>Đã hoàn thành</t>
+        </is>
       </c>
       <c r="O27" s="9" t="n">
-        <v>0.5</v>
+        <v>1.0</v>
       </c>
       <c r="P27" s="10" t="s">
         <v>323</v>
@@ -5001,11 +5049,13 @@
       <c r="M28" s="3" t="s">
         <v>328</v>
       </c>
-      <c r="N28" s="3" t="s">
-        <v>199</v>
+      <c r="N28" s="3" t="inlineStr">
+        <is>
+          <t>Đã hoàn thành</t>
+        </is>
       </c>
       <c r="O28" s="9" t="n">
-        <v>0</v>
+        <v>1.0</v>
       </c>
       <c r="P28" s="10" t="s">
         <v>329</v>
@@ -5051,11 +5101,13 @@
       <c r="M29" s="3" t="s">
         <v>334</v>
       </c>
-      <c r="N29" s="3" t="s">
-        <v>186</v>
+      <c r="N29" s="3" t="inlineStr">
+        <is>
+          <t>Đã hoàn thành</t>
+        </is>
       </c>
       <c r="O29" s="9" t="n">
-        <v>0.6</v>
+        <v>1.0</v>
       </c>
       <c r="P29" s="10" t="s">
         <v>335</v>
@@ -5101,11 +5153,13 @@
       <c r="M30" s="3" t="s">
         <v>340</v>
       </c>
-      <c r="N30" s="3" t="s">
-        <v>186</v>
+      <c r="N30" s="3" t="inlineStr">
+        <is>
+          <t>Đã hoàn thành</t>
+        </is>
       </c>
       <c r="O30" s="9" t="n">
-        <v>0.5</v>
+        <v>1.0</v>
       </c>
       <c r="P30" s="10" t="s">
         <v>341</v>
@@ -5151,11 +5205,13 @@
       <c r="M31" s="3" t="s">
         <v>346</v>
       </c>
-      <c r="N31" s="3" t="s">
-        <v>186</v>
+      <c r="N31" s="3" t="inlineStr">
+        <is>
+          <t>Đã hoàn thành</t>
+        </is>
       </c>
       <c r="O31" s="9" t="n">
-        <v>0.3</v>
+        <v>1.0</v>
       </c>
       <c r="P31" s="10" t="s">
         <v>347</v>
@@ -5201,11 +5257,13 @@
       <c r="M32" s="3" t="s">
         <v>352</v>
       </c>
-      <c r="N32" s="3" t="s">
-        <v>199</v>
+      <c r="N32" s="3" t="inlineStr">
+        <is>
+          <t>Đã hoàn thành</t>
+        </is>
       </c>
       <c r="O32" s="9" t="n">
-        <v>0</v>
+        <v>1.0</v>
       </c>
       <c r="P32" s="10" t="s">
         <v>353</v>
@@ -5251,11 +5309,13 @@
       <c r="M33" s="3" t="s">
         <v>358</v>
       </c>
-      <c r="N33" s="3" t="s">
-        <v>199</v>
+      <c r="N33" s="3" t="inlineStr">
+        <is>
+          <t>Đã hoàn thành</t>
+        </is>
       </c>
       <c r="O33" s="9" t="n">
-        <v>0</v>
+        <v>1.0</v>
       </c>
       <c r="P33" s="10" t="s">
         <v>359</v>
@@ -5301,11 +5361,13 @@
       <c r="M34" s="3" t="s">
         <v>364</v>
       </c>
-      <c r="N34" s="3" t="s">
-        <v>186</v>
+      <c r="N34" s="3" t="inlineStr">
+        <is>
+          <t>Đã hoàn thành</t>
+        </is>
       </c>
       <c r="O34" s="9" t="n">
-        <v>0.6</v>
+        <v>1.0</v>
       </c>
       <c r="P34" s="10" t="s">
         <v>365</v>
@@ -5351,11 +5413,13 @@
       <c r="M35" s="3" t="s">
         <v>370</v>
       </c>
-      <c r="N35" s="3" t="s">
-        <v>186</v>
+      <c r="N35" s="3" t="inlineStr">
+        <is>
+          <t>Đã hoàn thành</t>
+        </is>
       </c>
       <c r="O35" s="9" t="n">
-        <v>0.6</v>
+        <v>1.0</v>
       </c>
       <c r="P35" s="10" t="s">
         <v>371</v>
@@ -5401,11 +5465,13 @@
       <c r="M36" s="3" t="s">
         <v>376</v>
       </c>
-      <c r="N36" s="3" t="s">
-        <v>186</v>
+      <c r="N36" s="3" t="inlineStr">
+        <is>
+          <t>Đã hoàn thành</t>
+        </is>
       </c>
       <c r="O36" s="9" t="n">
-        <v>0.4</v>
+        <v>1.0</v>
       </c>
       <c r="P36" s="10" t="s">
         <v>377</v>
@@ -5451,11 +5517,13 @@
       <c r="M37" s="3" t="s">
         <v>382</v>
       </c>
-      <c r="N37" s="3" t="s">
-        <v>199</v>
+      <c r="N37" s="3" t="inlineStr">
+        <is>
+          <t>Đã hoàn thành</t>
+        </is>
       </c>
       <c r="O37" s="9" t="n">
-        <v>0</v>
+        <v>1.0</v>
       </c>
       <c r="P37" s="10" t="s">
         <v>229</v>
@@ -5501,11 +5569,13 @@
       <c r="M38" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="N38" s="3" t="s">
-        <v>186</v>
+      <c r="N38" s="3" t="inlineStr">
+        <is>
+          <t>Đã hoàn thành</t>
+        </is>
       </c>
       <c r="O38" s="9" t="n">
-        <v>0.6</v>
+        <v>1.0</v>
       </c>
       <c r="P38" s="10" t="s">
         <v>388</v>
@@ -5551,11 +5621,13 @@
       <c r="M39" s="3" t="s">
         <v>393</v>
       </c>
-      <c r="N39" s="3" t="s">
-        <v>186</v>
+      <c r="N39" s="3" t="inlineStr">
+        <is>
+          <t>Đã hoàn thành</t>
+        </is>
       </c>
       <c r="O39" s="9" t="n">
-        <v>0.3</v>
+        <v>1.0</v>
       </c>
       <c r="P39" s="10" t="s">
         <v>394</v>
@@ -5601,11 +5673,13 @@
       <c r="M40" s="3" t="s">
         <v>399</v>
       </c>
-      <c r="N40" s="3" t="s">
-        <v>199</v>
+      <c r="N40" s="3" t="inlineStr">
+        <is>
+          <t>Bị chặn</t>
+        </is>
       </c>
       <c r="O40" s="9" t="n">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="P40" s="10" t="s">
         <v>229</v>
@@ -5651,11 +5725,13 @@
       <c r="M41" s="3" t="s">
         <v>403</v>
       </c>
-      <c r="N41" s="3" t="s">
-        <v>199</v>
+      <c r="N41" s="3" t="inlineStr">
+        <is>
+          <t>Đã hoàn thành</t>
+        </is>
       </c>
       <c r="O41" s="9" t="n">
-        <v>0</v>
+        <v>1.0</v>
       </c>
       <c r="P41" s="10" t="s">
         <v>404</v>
@@ -5951,11 +6027,13 @@
       <c r="M47" s="3" t="s">
         <v>435</v>
       </c>
-      <c r="N47" s="3" t="s">
-        <v>199</v>
+      <c r="N47" s="3" t="inlineStr">
+        <is>
+          <t>Đã hoàn thành</t>
+        </is>
       </c>
       <c r="O47" s="9" t="n">
-        <v>0</v>
+        <v>1.0</v>
       </c>
       <c r="P47" s="10" t="s">
         <v>436</v>
@@ -6001,11 +6079,13 @@
       <c r="M48" s="3" t="s">
         <v>441</v>
       </c>
-      <c r="N48" s="3" t="s">
-        <v>199</v>
+      <c r="N48" s="3" t="inlineStr">
+        <is>
+          <t>Đã hoàn thành</t>
+        </is>
       </c>
       <c r="O48" s="9" t="n">
-        <v>0</v>
+        <v>1.0</v>
       </c>
       <c r="P48" s="10" t="s">
         <v>442</v>
@@ -6051,11 +6131,13 @@
       <c r="M49" s="3" t="s">
         <v>446</v>
       </c>
-      <c r="N49" s="3" t="s">
-        <v>199</v>
+      <c r="N49" s="3" t="inlineStr">
+        <is>
+          <t>Đã hoàn thành</t>
+        </is>
       </c>
       <c r="O49" s="9" t="n">
-        <v>0</v>
+        <v>1.0</v>
       </c>
       <c r="P49" s="10" t="s">
         <v>447</v>
@@ -6101,11 +6183,13 @@
       <c r="M50" s="3" t="s">
         <v>451</v>
       </c>
-      <c r="N50" s="3" t="s">
-        <v>199</v>
+      <c r="N50" s="3" t="inlineStr">
+        <is>
+          <t>Bị chặn</t>
+        </is>
       </c>
       <c r="O50" s="9" t="n">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="P50" s="10" t="s">
         <v>452</v>
@@ -6151,11 +6235,13 @@
       <c r="M51" s="3" t="s">
         <v>457</v>
       </c>
-      <c r="N51" s="3" t="s">
-        <v>199</v>
+      <c r="N51" s="3" t="inlineStr">
+        <is>
+          <t>Đang thực hiện</t>
+        </is>
       </c>
       <c r="O51" s="9" t="n">
-        <v>0</v>
+        <v>0.9</v>
       </c>
       <c r="P51" s="10" t="s">
         <v>229</v>
@@ -6201,11 +6287,13 @@
       <c r="M52" s="3" t="s">
         <v>463</v>
       </c>
-      <c r="N52" s="3" t="s">
-        <v>199</v>
+      <c r="N52" s="3" t="inlineStr">
+        <is>
+          <t>Đã hoàn thành</t>
+        </is>
       </c>
       <c r="O52" s="9" t="n">
-        <v>0</v>
+        <v>1.0</v>
       </c>
       <c r="P52" s="10" t="s">
         <v>464</v>
@@ -6251,11 +6339,13 @@
       <c r="M53" s="3" t="s">
         <v>468</v>
       </c>
-      <c r="N53" s="3" t="s">
-        <v>199</v>
+      <c r="N53" s="3" t="inlineStr">
+        <is>
+          <t>Bị chặn</t>
+        </is>
       </c>
       <c r="O53" s="9" t="n">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="P53" s="10" t="s">
         <v>469</v>
@@ -6301,11 +6391,13 @@
       <c r="M54" s="3" t="s">
         <v>474</v>
       </c>
-      <c r="N54" s="3" t="s">
-        <v>199</v>
+      <c r="N54" s="3" t="inlineStr">
+        <is>
+          <t>Đang thực hiện</t>
+        </is>
       </c>
       <c r="O54" s="9" t="n">
-        <v>0</v>
+        <v>0.85</v>
       </c>
       <c r="P54" s="10" t="s">
         <v>187</v>

</xml_diff>